<commit_message>
Add SOH report for 2026-10-31
</commit_message>
<xml_diff>
--- a/reports/SOH_31_10_2026.xlsx
+++ b/reports/SOH_31_10_2026.xlsx
@@ -9074,7 +9074,7 @@
         </is>
       </c>
       <c r="D312" s="2" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E312" s="3" t="n">
         <v>1</v>
@@ -9410,7 +9410,7 @@
         </is>
       </c>
       <c r="D324" s="2" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E324" s="3" t="n">
         <v>1</v>
@@ -10586,7 +10586,7 @@
         </is>
       </c>
       <c r="D366" s="2" t="n">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="E366" s="3" t="n">
         <v>8000</v>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="D377" s="2" t="n">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E377" s="3" t="n">
         <v>40000</v>
@@ -11622,7 +11622,7 @@
         </is>
       </c>
       <c r="D403" s="2" t="n">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E403" s="3" t="n">
         <v>81000</v>
@@ -12014,7 +12014,7 @@
         </is>
       </c>
       <c r="D417" s="2" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E417" s="3" t="n">
         <v>8000</v>
@@ -12042,7 +12042,7 @@
         </is>
       </c>
       <c r="D418" s="2" t="n">
-        <v>1295</v>
+        <v>1289</v>
       </c>
       <c r="E418" s="3" t="n">
         <v>8000</v>
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="D419" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E419" s="3" t="n">
         <v>10000</v>
@@ -12098,7 +12098,7 @@
         </is>
       </c>
       <c r="D420" s="2" t="n">
-        <v>-59</v>
+        <v>-65</v>
       </c>
       <c r="E420" s="3" t="n">
         <v>8000</v>
@@ -12154,7 +12154,7 @@
         </is>
       </c>
       <c r="D422" s="2" t="n">
-        <v>-68</v>
+        <v>-74</v>
       </c>
       <c r="E422" s="3" t="n">
         <v>8000</v>
@@ -12210,7 +12210,7 @@
         </is>
       </c>
       <c r="D424" s="2" t="n">
-        <v>-70</v>
+        <v>-76</v>
       </c>
       <c r="E424" s="3" t="n">
         <v>8000</v>
@@ -18874,7 +18874,7 @@
         </is>
       </c>
       <c r="D662" s="2" t="n">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E662" s="3" t="n">
         <v>1</v>
@@ -20414,7 +20414,7 @@
         </is>
       </c>
       <c r="D717" s="2" t="n">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E717" s="3" t="n">
         <v>1</v>
@@ -25650,7 +25650,7 @@
         </is>
       </c>
       <c r="D904" s="2" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E904" s="3" t="n">
         <v>1</v>
@@ -26098,7 +26098,7 @@
         </is>
       </c>
       <c r="D920" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E920" s="3" t="n">
         <v>13734</v>
@@ -26154,7 +26154,7 @@
         </is>
       </c>
       <c r="D922" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E922" s="3" t="n">
         <v>18059</v>

</xml_diff>